<commit_message>
in this i have include the interface to deploy:
</commit_message>
<xml_diff>
--- a/final.xlsx
+++ b/final.xlsx
@@ -527,7 +527,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.919892857142857</v>
+        <v>0.9198928571428572</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>1</v>
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0.5542500000000001</v>
+        <v>0.55425</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>0</v>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.7790573593073593</v>
+        <v>0.7790573593073594</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>1</v>
@@ -846,7 +846,7 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0.4272241245344695</v>
+        <v>0.4272241245344693</v>
       </c>
       <c r="F14" s="2" t="n">
         <v>0</v>
@@ -904,7 +904,7 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0.7223377100840337</v>
+        <v>0.7223377100840335</v>
       </c>
       <c r="F16" s="2" t="n">
         <v>1</v>
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0.6320456349206349</v>
+        <v>0.6320456349206348</v>
       </c>
       <c r="F18" s="2" t="n">
         <v>0</v>
@@ -991,7 +991,7 @@
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>0.6422142857142856</v>
+        <v>0.6422142857142857</v>
       </c>
       <c r="F19" s="2" t="n">
         <v>1</v>
@@ -1049,7 +1049,7 @@
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>0.843678223555089</v>
+        <v>0.8436782235550889</v>
       </c>
       <c r="F21" s="2" t="n">
         <v>1</v>
@@ -1078,7 +1078,7 @@
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>0.04054166666666666</v>
+        <v>0.04054166666666667</v>
       </c>
       <c r="F22" s="2" t="n">
         <v>0</v>
@@ -1136,7 +1136,7 @@
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0.9718511904761905</v>
+        <v>0.9718511904761904</v>
       </c>
       <c r="F24" s="2" t="n">
         <v>1</v>
@@ -1223,7 +1223,7 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.9278387836661068</v>
+        <v>0.9278387836661069</v>
       </c>
       <c r="F27" s="2" t="n">
         <v>1</v>
@@ -1339,7 +1339,7 @@
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0.4018544127788496</v>
+        <v>0.4018544127788497</v>
       </c>
       <c r="F31" s="2" t="n">
         <v>0</v>
@@ -1397,7 +1397,7 @@
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>0.9069393939393936</v>
+        <v>0.9069393939393937</v>
       </c>
       <c r="F33" s="2" t="n">
         <v>1</v>
@@ -1426,7 +1426,7 @@
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>0.6894469779377966</v>
+        <v>0.6894469779377965</v>
       </c>
       <c r="F34" s="2" t="n">
         <v>0</v>
@@ -1629,7 +1629,7 @@
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>0.3399492722190091</v>
+        <v>0.339949272219009</v>
       </c>
       <c r="F41" s="2" t="n">
         <v>0</v>
@@ -1803,7 +1803,7 @@
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0.8232261904761906</v>
+        <v>0.8232261904761907</v>
       </c>
       <c r="F47" s="2" t="n">
         <v>1</v>
@@ -1890,7 +1890,7 @@
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>0.5906914362519201</v>
+        <v>0.59069143625192</v>
       </c>
       <c r="F50" s="2" t="n">
         <v>1</v>
@@ -1977,7 +1977,7 @@
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>0.6680634920634921</v>
+        <v>0.6680634920634919</v>
       </c>
       <c r="F53" s="2" t="n">
         <v>0</v>
@@ -2006,7 +2006,7 @@
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>0.5234505175525537</v>
+        <v>0.5234505175525538</v>
       </c>
       <c r="F54" s="2" t="n">
         <v>0</v>
@@ -2122,7 +2122,7 @@
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>0.9765714285714284</v>
+        <v>0.9765714285714285</v>
       </c>
       <c r="F58" s="2" t="n">
         <v>1</v>
@@ -2412,7 +2412,7 @@
         </is>
       </c>
       <c r="E68" s="2" t="n">
-        <v>0.4414920634920635</v>
+        <v>0.4414920634920634</v>
       </c>
       <c r="F68" s="2" t="n">
         <v>0</v>
@@ -2586,7 +2586,7 @@
         </is>
       </c>
       <c r="E74" s="2" t="n">
-        <v>0.596576296510507</v>
+        <v>0.5965762965105069</v>
       </c>
       <c r="F74" s="2" t="n">
         <v>0</v>
@@ -2644,7 +2644,7 @@
         </is>
       </c>
       <c r="E76" s="2" t="n">
-        <v>0.6708056247553447</v>
+        <v>0.6708056247553444</v>
       </c>
       <c r="F76" s="2" t="n">
         <v>0</v>
@@ -2731,7 +2731,7 @@
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>0.9517083333333334</v>
+        <v>0.9517083333333335</v>
       </c>
       <c r="F79" s="2" t="n">
         <v>1</v>
@@ -2760,7 +2760,7 @@
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>0.3934880952380952</v>
+        <v>0.3934880952380953</v>
       </c>
       <c r="F80" s="2" t="n">
         <v>0</v>
@@ -2818,7 +2818,7 @@
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>0.5880358226976869</v>
+        <v>0.5880358226976868</v>
       </c>
       <c r="F82" s="2" t="n">
         <v>0</v>
@@ -2963,7 +2963,7 @@
         </is>
       </c>
       <c r="E87" s="2" t="n">
-        <v>0.5606511033084481</v>
+        <v>0.560651103308448</v>
       </c>
       <c r="F87" s="2" t="n">
         <v>0</v>
@@ -3079,7 +3079,7 @@
         </is>
       </c>
       <c r="E91" s="2" t="n">
-        <v>0.8154085497835498</v>
+        <v>0.8154085497835497</v>
       </c>
       <c r="F91" s="2" t="n">
         <v>1</v>
@@ -3195,7 +3195,7 @@
         </is>
       </c>
       <c r="E95" s="2" t="n">
-        <v>0.8660094161958569</v>
+        <v>0.8660094161958568</v>
       </c>
       <c r="F95" s="2" t="n">
         <v>1</v>
@@ -3369,7 +3369,7 @@
         </is>
       </c>
       <c r="E101" s="2" t="n">
-        <v>0.7105624910043068</v>
+        <v>0.7105624910043069</v>
       </c>
       <c r="F101" s="2" t="n">
         <v>1</v>
@@ -3398,7 +3398,7 @@
         </is>
       </c>
       <c r="E102" s="2" t="n">
-        <v>0.6048670634920634</v>
+        <v>0.6048670634920635</v>
       </c>
       <c r="F102" s="2" t="n">
         <v>1</v>
@@ -3514,7 +3514,7 @@
         </is>
       </c>
       <c r="E106" s="2" t="n">
-        <v>0.9835967578520771</v>
+        <v>0.983596757852077</v>
       </c>
       <c r="F106" s="2" t="n">
         <v>1</v>
@@ -3601,7 +3601,7 @@
         </is>
       </c>
       <c r="E109" s="2" t="n">
-        <v>0.7049858733157265</v>
+        <v>0.7049858733157266</v>
       </c>
       <c r="F109" s="2" t="n">
         <v>0</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="E110" s="2" t="n">
-        <v>0.6829029458479104</v>
+        <v>0.6829029458479102</v>
       </c>
       <c r="F110" s="2" t="n">
         <v>0</v>
@@ -3804,7 +3804,7 @@
         </is>
       </c>
       <c r="E116" s="2" t="n">
-        <v>0.6724025141525142</v>
+        <v>0.6724025141525144</v>
       </c>
       <c r="F116" s="2" t="n">
         <v>1</v>
@@ -4123,7 +4123,7 @@
         </is>
       </c>
       <c r="E127" s="2" t="n">
-        <v>0.4310990849273632</v>
+        <v>0.4310990849273633</v>
       </c>
       <c r="F127" s="2" t="n">
         <v>0</v>
@@ -4297,7 +4297,7 @@
         </is>
       </c>
       <c r="E133" s="2" t="n">
-        <v>0.8640465132818075</v>
+        <v>0.8640465132818076</v>
       </c>
       <c r="F133" s="2" t="n">
         <v>1</v>
@@ -4442,7 +4442,7 @@
         </is>
       </c>
       <c r="E138" s="2" t="n">
-        <v>0.5993988095238095</v>
+        <v>0.5993988095238096</v>
       </c>
       <c r="F138" s="2" t="n">
         <v>1</v>
@@ -4645,7 +4645,7 @@
         </is>
       </c>
       <c r="E145" s="2" t="n">
-        <v>0.8174654070414621</v>
+        <v>0.817465407041462</v>
       </c>
       <c r="F145" s="2" t="n">
         <v>1</v>
@@ -4819,7 +4819,7 @@
         </is>
       </c>
       <c r="E151" s="2" t="n">
-        <v>0.2133035714285714</v>
+        <v>0.2133035714285715</v>
       </c>
       <c r="F151" s="2" t="n">
         <v>0</v>
@@ -4848,7 +4848,7 @@
         </is>
       </c>
       <c r="E152" s="2" t="n">
-        <v>0.8486726190476189</v>
+        <v>0.8486726190476187</v>
       </c>
       <c r="F152" s="2" t="n">
         <v>1</v>
@@ -4906,7 +4906,7 @@
         </is>
       </c>
       <c r="E154" s="2" t="n">
-        <v>0.6469685845758795</v>
+        <v>0.6469685845758794</v>
       </c>
       <c r="F154" s="2" t="n">
         <v>0</v>
@@ -4935,7 +4935,7 @@
         </is>
       </c>
       <c r="E155" s="2" t="n">
-        <v>0.4968274853801171</v>
+        <v>0.496827485380117</v>
       </c>
       <c r="F155" s="2" t="n">
         <v>1</v>
@@ -5138,7 +5138,7 @@
         </is>
       </c>
       <c r="E162" s="2" t="n">
-        <v>0.5779795875421172</v>
+        <v>0.5779795875421173</v>
       </c>
       <c r="F162" s="2" t="n">
         <v>0</v>
@@ -5196,7 +5196,7 @@
         </is>
       </c>
       <c r="E164" s="2" t="n">
-        <v>0.9423195488721805</v>
+        <v>0.9423195488721804</v>
       </c>
       <c r="F164" s="2" t="n">
         <v>1</v>
@@ -5399,7 +5399,7 @@
         </is>
       </c>
       <c r="E171" s="2" t="n">
-        <v>0.5627748867763332</v>
+        <v>0.5627748867763334</v>
       </c>
       <c r="F171" s="2" t="n">
         <v>0</v>
@@ -5602,7 +5602,7 @@
         </is>
       </c>
       <c r="E178" s="2" t="n">
-        <v>0.3704009740259741</v>
+        <v>0.3704009740259739</v>
       </c>
       <c r="F178" s="2" t="n">
         <v>1</v>
@@ -5631,7 +5631,7 @@
         </is>
       </c>
       <c r="E179" s="2" t="n">
-        <v>0.6794880952380953</v>
+        <v>0.6844880952380954</v>
       </c>
       <c r="F179" s="2" t="n">
         <v>1</v>
@@ -5718,7 +5718,7 @@
         </is>
       </c>
       <c r="E182" s="2" t="n">
-        <v>0.3994332444041746</v>
+        <v>0.3994332444041745</v>
       </c>
       <c r="F182" s="2" t="n">
         <v>0</v>
@@ -5776,7 +5776,7 @@
         </is>
       </c>
       <c r="E184" s="2" t="n">
-        <v>0.03167857142857142</v>
+        <v>0.03167857142857143</v>
       </c>
       <c r="F184" s="2" t="n">
         <v>0</v>
@@ -5834,7 +5834,7 @@
         </is>
       </c>
       <c r="E186" s="2" t="n">
-        <v>0.7622805111555111</v>
+        <v>0.7622805111555112</v>
       </c>
       <c r="F186" s="2" t="n">
         <v>1</v>
@@ -5892,7 +5892,7 @@
         </is>
       </c>
       <c r="E188" s="2" t="n">
-        <v>0.8665550695124022</v>
+        <v>0.8665550695124025</v>
       </c>
       <c r="F188" s="2" t="n">
         <v>1</v>
@@ -5921,7 +5921,7 @@
         </is>
       </c>
       <c r="E189" s="2" t="n">
-        <v>0.9126444778389826</v>
+        <v>0.9126444778389825</v>
       </c>
       <c r="F189" s="2" t="n">
         <v>1</v>
@@ -6008,7 +6008,7 @@
         </is>
       </c>
       <c r="E192" s="2" t="n">
-        <v>0.482779676463887</v>
+        <v>0.4827796764638869</v>
       </c>
       <c r="F192" s="2" t="n">
         <v>1</v>
@@ -6095,7 +6095,7 @@
         </is>
       </c>
       <c r="E195" s="2" t="n">
-        <v>0.8994473443223441</v>
+        <v>0.899447344322344</v>
       </c>
       <c r="F195" s="2" t="n">
         <v>1</v>
@@ -6124,7 +6124,7 @@
         </is>
       </c>
       <c r="E196" s="2" t="n">
-        <v>0.02558333333333334</v>
+        <v>0.02558333333333333</v>
       </c>
       <c r="F196" s="2" t="n">
         <v>0</v>
@@ -6153,7 +6153,7 @@
         </is>
       </c>
       <c r="E197" s="2" t="n">
-        <v>0.9518817443286326</v>
+        <v>0.9518817443286328</v>
       </c>
       <c r="F197" s="2" t="n">
         <v>1</v>
@@ -6414,7 +6414,7 @@
         </is>
       </c>
       <c r="E206" s="2" t="n">
-        <v>0.6619890389751238</v>
+        <v>0.6619890389751236</v>
       </c>
       <c r="F206" s="2" t="n">
         <v>1</v>
@@ -6472,7 +6472,7 @@
         </is>
       </c>
       <c r="E208" s="2" t="n">
-        <v>0.872123015873016</v>
+        <v>0.8721230158730158</v>
       </c>
       <c r="F208" s="2" t="n">
         <v>1</v>
@@ -6646,7 +6646,7 @@
         </is>
       </c>
       <c r="E214" s="2" t="n">
-        <v>0.9601079291079293</v>
+        <v>0.9601079291079292</v>
       </c>
       <c r="F214" s="2" t="n">
         <v>1</v>
@@ -6733,7 +6733,7 @@
         </is>
       </c>
       <c r="E217" s="2" t="n">
-        <v>0.6716825396825397</v>
+        <v>0.6716825396825395</v>
       </c>
       <c r="F217" s="2" t="n">
         <v>1</v>
@@ -7197,7 +7197,7 @@
         </is>
       </c>
       <c r="E233" s="2" t="n">
-        <v>0.9160651966137884</v>
+        <v>0.9160651966137885</v>
       </c>
       <c r="F233" s="2" t="n">
         <v>1</v>
@@ -7255,7 +7255,7 @@
         </is>
       </c>
       <c r="E235" s="2" t="n">
-        <v>0.5530057110796845</v>
+        <v>0.5530057110796847</v>
       </c>
       <c r="F235" s="2" t="n">
         <v>0</v>
@@ -7342,7 +7342,7 @@
         </is>
       </c>
       <c r="E238" s="2" t="n">
-        <v>0.6661658158277768</v>
+        <v>0.6661658158277767</v>
       </c>
       <c r="F238" s="2" t="n">
         <v>0</v>
@@ -7400,7 +7400,7 @@
         </is>
       </c>
       <c r="E240" s="2" t="n">
-        <v>0.608874633615452</v>
+        <v>0.6088746336154521</v>
       </c>
       <c r="F240" s="2" t="n">
         <v>1</v>
@@ -7487,7 +7487,7 @@
         </is>
       </c>
       <c r="E243" s="2" t="n">
-        <v>0.839261904761905</v>
+        <v>0.8392619047619051</v>
       </c>
       <c r="F243" s="2" t="n">
         <v>1</v>
@@ -7603,7 +7603,7 @@
         </is>
       </c>
       <c r="E247" s="2" t="n">
-        <v>0.697139194139194</v>
+        <v>0.6971391941391941</v>
       </c>
       <c r="F247" s="2" t="n">
         <v>0</v>
@@ -7632,7 +7632,7 @@
         </is>
       </c>
       <c r="E248" s="2" t="n">
-        <v>0.8119999999999998</v>
+        <v>0.8120000000000001</v>
       </c>
       <c r="F248" s="2" t="n">
         <v>0</v>
@@ -7748,7 +7748,7 @@
         </is>
       </c>
       <c r="E252" s="2" t="n">
-        <v>0.06268849206349207</v>
+        <v>0.06268849206349206</v>
       </c>
       <c r="F252" s="2" t="n">
         <v>0</v>
@@ -7922,7 +7922,7 @@
         </is>
       </c>
       <c r="E258" s="2" t="n">
-        <v>0.1975357142857144</v>
+        <v>0.1975357142857143</v>
       </c>
       <c r="F258" s="2" t="n">
         <v>0</v>
@@ -7951,7 +7951,7 @@
         </is>
       </c>
       <c r="E259" s="2" t="n">
-        <v>0.4790833333333333</v>
+        <v>0.4790833333333332</v>
       </c>
       <c r="F259" s="2" t="n">
         <v>0</v>
@@ -8096,7 +8096,7 @@
         </is>
       </c>
       <c r="E264" s="2" t="n">
-        <v>0.8344354448233758</v>
+        <v>0.8344354448233759</v>
       </c>
       <c r="F264" s="2" t="n">
         <v>1</v>
@@ -8241,7 +8241,7 @@
         </is>
       </c>
       <c r="E269" s="2" t="n">
-        <v>0.4742086601075958</v>
+        <v>0.4742086601075957</v>
       </c>
       <c r="F269" s="2" t="n">
         <v>1</v>
@@ -8328,7 +8328,7 @@
         </is>
       </c>
       <c r="E272" s="2" t="n">
-        <v>0.4084215949820789</v>
+        <v>0.4084215949820788</v>
       </c>
       <c r="F272" s="2" t="n">
         <v>1</v>
@@ -8415,7 +8415,7 @@
         </is>
       </c>
       <c r="E275" s="2" t="n">
-        <v>0.6685190035450161</v>
+        <v>0.6685190035450159</v>
       </c>
       <c r="F275" s="2" t="n">
         <v>1</v>
@@ -8705,7 +8705,7 @@
         </is>
       </c>
       <c r="E285" s="2" t="n">
-        <v>0.6743902723959663</v>
+        <v>0.6743902723959662</v>
       </c>
       <c r="F285" s="2" t="n">
         <v>0</v>
@@ -8763,7 +8763,7 @@
         </is>
       </c>
       <c r="E287" s="2" t="n">
-        <v>0.8301188566335624</v>
+        <v>0.8301188566335626</v>
       </c>
       <c r="F287" s="2" t="n">
         <v>0</v>
@@ -8850,7 +8850,7 @@
         </is>
       </c>
       <c r="E290" s="2" t="n">
-        <v>0.04219444444444445</v>
+        <v>0.04219444444444444</v>
       </c>
       <c r="F290" s="2" t="n">
         <v>0</v>
@@ -9140,7 +9140,7 @@
         </is>
       </c>
       <c r="E300" s="2" t="n">
-        <v>0.7753134920634921</v>
+        <v>0.7753134920634919</v>
       </c>
       <c r="F300" s="2" t="n">
         <v>1</v>
@@ -9169,7 +9169,7 @@
         </is>
       </c>
       <c r="E301" s="2" t="n">
-        <v>0.4191488095238097</v>
+        <v>0.4191488095238096</v>
       </c>
       <c r="F301" s="2" t="n">
         <v>0</v>
@@ -9285,7 +9285,7 @@
         </is>
       </c>
       <c r="E305" s="2" t="n">
-        <v>0.7095952380952381</v>
+        <v>0.7095952380952382</v>
       </c>
       <c r="F305" s="2" t="n">
         <v>1</v>
@@ -9691,7 +9691,7 @@
         </is>
       </c>
       <c r="E319" s="2" t="n">
-        <v>0.8637788387087167</v>
+        <v>0.8637788387087169</v>
       </c>
       <c r="F319" s="2" t="n">
         <v>1</v>
@@ -9749,7 +9749,7 @@
         </is>
       </c>
       <c r="E321" s="2" t="n">
-        <v>0.4364983563413098</v>
+        <v>0.4364983563413097</v>
       </c>
       <c r="F321" s="2" t="n">
         <v>0</v>
@@ -9894,7 +9894,7 @@
         </is>
       </c>
       <c r="E326" s="2" t="n">
-        <v>0.9597500000000001</v>
+        <v>0.95975</v>
       </c>
       <c r="F326" s="2" t="n">
         <v>1</v>
@@ -10039,7 +10039,7 @@
         </is>
       </c>
       <c r="E331" s="2" t="n">
-        <v>0.07630357142857143</v>
+        <v>0.07630357142857144</v>
       </c>
       <c r="F331" s="2" t="n">
         <v>0</v>
@@ -10068,7 +10068,7 @@
         </is>
       </c>
       <c r="E332" s="2" t="n">
-        <v>0.8568998917748918</v>
+        <v>0.856899891774892</v>
       </c>
       <c r="F332" s="2" t="n">
         <v>1</v>
@@ -10271,7 +10271,7 @@
         </is>
       </c>
       <c r="E339" s="2" t="n">
-        <v>0.8820476190476186</v>
+        <v>0.882047619047619</v>
       </c>
       <c r="F339" s="2" t="n">
         <v>1</v>
@@ -10416,7 +10416,7 @@
         </is>
       </c>
       <c r="E344" s="2" t="n">
-        <v>0.5057460032657402</v>
+        <v>0.50574600326574</v>
       </c>
       <c r="F344" s="2" t="n">
         <v>0</v>
@@ -10619,7 +10619,7 @@
         </is>
       </c>
       <c r="E351" s="2" t="n">
-        <v>0.8756476885715171</v>
+        <v>0.8756476885715172</v>
       </c>
       <c r="F351" s="2" t="n">
         <v>1</v>
@@ -10677,7 +10677,7 @@
         </is>
       </c>
       <c r="E353" s="2" t="n">
-        <v>0.8081017666434827</v>
+        <v>0.8081017666434828</v>
       </c>
       <c r="F353" s="2" t="n">
         <v>0</v>
@@ -10793,7 +10793,7 @@
         </is>
       </c>
       <c r="E357" s="2" t="n">
-        <v>0.8958363021387215</v>
+        <v>0.8958363021387216</v>
       </c>
       <c r="F357" s="2" t="n">
         <v>1</v>
@@ -11170,7 +11170,7 @@
         </is>
       </c>
       <c r="E370" s="2" t="n">
-        <v>0.4377460317460319</v>
+        <v>0.4377460317460317</v>
       </c>
       <c r="F370" s="2" t="n">
         <v>0</v>
@@ -11257,7 +11257,7 @@
         </is>
       </c>
       <c r="E373" s="2" t="n">
-        <v>0.9054804639804638</v>
+        <v>0.905480463980464</v>
       </c>
       <c r="F373" s="2" t="n">
         <v>1</v>
@@ -11547,7 +11547,7 @@
         </is>
       </c>
       <c r="E383" s="2" t="n">
-        <v>0.3735677655677656</v>
+        <v>0.3735677655677655</v>
       </c>
       <c r="F383" s="2" t="n">
         <v>0</v>
@@ -11576,7 +11576,7 @@
         </is>
       </c>
       <c r="E384" s="2" t="n">
-        <v>0.9130904845169396</v>
+        <v>0.9130904845169395</v>
       </c>
       <c r="F384" s="2" t="n">
         <v>1</v>
@@ -11634,7 +11634,7 @@
         </is>
       </c>
       <c r="E386" s="2" t="n">
-        <v>0.3243989086571324</v>
+        <v>0.3243989086571323</v>
       </c>
       <c r="F386" s="2" t="n">
         <v>0</v>
@@ -11692,7 +11692,7 @@
         </is>
       </c>
       <c r="E388" s="2" t="n">
-        <v>0.7160604261382737</v>
+        <v>0.7160604261382736</v>
       </c>
       <c r="F388" s="2" t="n">
         <v>1</v>
@@ -11808,7 +11808,7 @@
         </is>
       </c>
       <c r="E392" s="2" t="n">
-        <v>0.6034642857142856</v>
+        <v>0.6034642857142857</v>
       </c>
       <c r="F392" s="2" t="n">
         <v>0</v>
@@ -11982,7 +11982,7 @@
         </is>
       </c>
       <c r="E398" s="2" t="n">
-        <v>0.3801314816397053</v>
+        <v>0.3801314816397054</v>
       </c>
       <c r="F398" s="2" t="n">
         <v>1</v>
@@ -12098,7 +12098,7 @@
         </is>
       </c>
       <c r="E402" s="2" t="n">
-        <v>0.3820288461538461</v>
+        <v>0.3820288461538462</v>
       </c>
       <c r="F402" s="2" t="n">
         <v>0</v>
@@ -12127,7 +12127,7 @@
         </is>
       </c>
       <c r="E403" s="2" t="n">
-        <v>0.8425714285714285</v>
+        <v>0.8425714285714286</v>
       </c>
       <c r="F403" s="2" t="n">
         <v>1</v>
@@ -12156,7 +12156,7 @@
         </is>
       </c>
       <c r="E404" s="2" t="n">
-        <v>0.5553973685628097</v>
+        <v>0.5553973685628099</v>
       </c>
       <c r="F404" s="2" t="n">
         <v>0</v>
@@ -12301,7 +12301,7 @@
         </is>
       </c>
       <c r="E409" s="2" t="n">
-        <v>0.8672261904761903</v>
+        <v>0.8672261904761904</v>
       </c>
       <c r="F409" s="2" t="n">
         <v>1</v>
@@ -12359,7 +12359,7 @@
         </is>
       </c>
       <c r="E411" s="2" t="n">
-        <v>0.8605618366505339</v>
+        <v>0.8638951699838671</v>
       </c>
       <c r="F411" s="2" t="n">
         <v>0</v>
@@ -12533,7 +12533,7 @@
         </is>
       </c>
       <c r="E417" s="2" t="n">
-        <v>0.7273632668964669</v>
+        <v>0.7273632668964667</v>
       </c>
       <c r="F417" s="2" t="n">
         <v>1</v>
@@ -12591,7 +12591,7 @@
         </is>
       </c>
       <c r="E419" s="2" t="n">
-        <v>0.7204350414078678</v>
+        <v>0.7204350414078676</v>
       </c>
       <c r="F419" s="2" t="n">
         <v>0</v>
@@ -12823,7 +12823,7 @@
         </is>
       </c>
       <c r="E427" s="2" t="n">
-        <v>0.05263888888888888</v>
+        <v>0.05263888888888889</v>
       </c>
       <c r="F427" s="2" t="n">
         <v>0</v>
@@ -12910,7 +12910,7 @@
         </is>
       </c>
       <c r="E430" s="2" t="n">
-        <v>0.4042936785436786</v>
+        <v>0.4042936785436787</v>
       </c>
       <c r="F430" s="2" t="n">
         <v>0</v>
@@ -13026,7 +13026,7 @@
         </is>
       </c>
       <c r="E434" s="2" t="n">
-        <v>0.9925084175084175</v>
+        <v>0.9925084175084176</v>
       </c>
       <c r="F434" s="2" t="n">
         <v>1</v>
@@ -13171,7 +13171,7 @@
         </is>
       </c>
       <c r="E439" s="2" t="n">
-        <v>0.4433062285777804</v>
+        <v>0.4433062285777805</v>
       </c>
       <c r="F439" s="2" t="n">
         <v>0</v>
@@ -13229,7 +13229,7 @@
         </is>
       </c>
       <c r="E441" s="2" t="n">
-        <v>0.7286475841321177</v>
+        <v>0.7286475841321176</v>
       </c>
       <c r="F441" s="2" t="n">
         <v>1</v>
@@ -13316,7 +13316,7 @@
         </is>
       </c>
       <c r="E444" s="2" t="n">
-        <v>0.7392593889847962</v>
+        <v>0.739259388984796</v>
       </c>
       <c r="F444" s="2" t="n">
         <v>1</v>
@@ -13374,7 +13374,7 @@
         </is>
       </c>
       <c r="E446" s="2" t="n">
-        <v>0.8705456349206347</v>
+        <v>0.870545634920635</v>
       </c>
       <c r="F446" s="2" t="n">
         <v>1</v>
@@ -13577,7 +13577,7 @@
         </is>
       </c>
       <c r="E453" s="2" t="n">
-        <v>0.8860829831932773</v>
+        <v>0.8860829831932775</v>
       </c>
       <c r="F453" s="2" t="n">
         <v>1</v>
@@ -13693,7 +13693,7 @@
         </is>
       </c>
       <c r="E457" s="2" t="n">
-        <v>0.584613095238095</v>
+        <v>0.5846130952380951</v>
       </c>
       <c r="F457" s="2" t="n">
         <v>0</v>
@@ -13780,7 +13780,7 @@
         </is>
       </c>
       <c r="E460" s="2" t="n">
-        <v>0.6175337301587303</v>
+        <v>0.6175337301587301</v>
       </c>
       <c r="F460" s="2" t="n">
         <v>0</v>
@@ -13896,7 +13896,7 @@
         </is>
       </c>
       <c r="E464" s="2" t="n">
-        <v>0.5818156565656564</v>
+        <v>0.5818156565656565</v>
       </c>
       <c r="F464" s="2" t="n">
         <v>1</v>
@@ -13954,7 +13954,7 @@
         </is>
       </c>
       <c r="E466" s="2" t="n">
-        <v>0.5161835598611917</v>
+        <v>0.5161835598611916</v>
       </c>
       <c r="F466" s="2" t="n">
         <v>1</v>
@@ -14041,7 +14041,7 @@
         </is>
       </c>
       <c r="E469" s="2" t="n">
-        <v>0.9838501027246227</v>
+        <v>0.9838501027246228</v>
       </c>
       <c r="F469" s="2" t="n">
         <v>1</v>
@@ -14476,7 +14476,7 @@
         </is>
       </c>
       <c r="E484" s="2" t="n">
-        <v>0.8351666666666665</v>
+        <v>0.8351666666666666</v>
       </c>
       <c r="F484" s="2" t="n">
         <v>1</v>
@@ -14563,7 +14563,7 @@
         </is>
       </c>
       <c r="E487" s="2" t="n">
-        <v>0.6641463585434174</v>
+        <v>0.6641463585434175</v>
       </c>
       <c r="F487" s="2" t="n">
         <v>1</v>
@@ -14679,7 +14679,7 @@
         </is>
       </c>
       <c r="E491" s="2" t="n">
-        <v>0.5832664332279242</v>
+        <v>0.583266433227924</v>
       </c>
       <c r="F491" s="2" t="n">
         <v>1</v>
@@ -14737,7 +14737,7 @@
         </is>
       </c>
       <c r="E493" s="2" t="n">
-        <v>0.6638928571428573</v>
+        <v>0.6638928571428572</v>
       </c>
       <c r="F493" s="2" t="n">
         <v>1</v>
@@ -14911,7 +14911,7 @@
         </is>
       </c>
       <c r="E499" s="2" t="n">
-        <v>0.8560586923805806</v>
+        <v>0.8560586923805805</v>
       </c>
       <c r="F499" s="2" t="n">
         <v>1</v>
@@ -15085,7 +15085,7 @@
         </is>
       </c>
       <c r="E505" s="2" t="n">
-        <v>0.9395654761904761</v>
+        <v>0.9395654761904763</v>
       </c>
       <c r="F505" s="2" t="n">
         <v>1</v>
@@ -15375,7 +15375,7 @@
         </is>
       </c>
       <c r="E515" s="2" t="n">
-        <v>0.8019551820728291</v>
+        <v>0.801955182072829</v>
       </c>
       <c r="F515" s="2" t="n">
         <v>1</v>
@@ -15491,7 +15491,7 @@
         </is>
       </c>
       <c r="E519" s="2" t="n">
-        <v>0.9213928571428573</v>
+        <v>0.9213928571428572</v>
       </c>
       <c r="F519" s="2" t="n">
         <v>0</v>
@@ -15549,7 +15549,7 @@
         </is>
       </c>
       <c r="E521" s="2" t="n">
-        <v>0.9798333333333333</v>
+        <v>0.9798333333333332</v>
       </c>
       <c r="F521" s="2" t="n">
         <v>0</v>
@@ -15723,7 +15723,7 @@
         </is>
       </c>
       <c r="E527" s="2" t="n">
-        <v>0.8671210317460316</v>
+        <v>0.8671210317460317</v>
       </c>
       <c r="F527" s="2" t="n">
         <v>1</v>
@@ -15955,7 +15955,7 @@
         </is>
       </c>
       <c r="E535" s="2" t="n">
-        <v>0.6605535714285713</v>
+        <v>0.6605535714285715</v>
       </c>
       <c r="F535" s="2" t="n">
         <v>0</v>
@@ -16303,7 +16303,7 @@
         </is>
       </c>
       <c r="E547" s="2" t="n">
-        <v>0.7006369047619049</v>
+        <v>0.7006369047619048</v>
       </c>
       <c r="F547" s="2" t="n">
         <v>1</v>
@@ -16477,7 +16477,7 @@
         </is>
       </c>
       <c r="E553" s="2" t="n">
-        <v>0.7206338074835898</v>
+        <v>0.7206338074835896</v>
       </c>
       <c r="F553" s="2" t="n">
         <v>1</v>
@@ -16651,7 +16651,7 @@
         </is>
       </c>
       <c r="E559" s="2" t="n">
-        <v>0.843513888888889</v>
+        <v>0.8435138888888888</v>
       </c>
       <c r="F559" s="2" t="n">
         <v>0</v>
@@ -16767,7 +16767,7 @@
         </is>
       </c>
       <c r="E563" s="2" t="n">
-        <v>0.6604461233211235</v>
+        <v>0.6604461233211234</v>
       </c>
       <c r="F563" s="2" t="n">
         <v>1</v>
@@ -16796,7 +16796,7 @@
         </is>
       </c>
       <c r="E564" s="2" t="n">
-        <v>0.5847886527176825</v>
+        <v>0.5847886527176823</v>
       </c>
       <c r="F564" s="2" t="n">
         <v>0</v>
@@ -16912,7 +16912,7 @@
         </is>
       </c>
       <c r="E568" s="2" t="n">
-        <v>0.3377092933947772</v>
+        <v>0.3377092933947773</v>
       </c>
       <c r="F568" s="2" t="n">
         <v>1</v>
@@ -17057,7 +17057,7 @@
         </is>
       </c>
       <c r="E573" s="2" t="n">
-        <v>0.8017251082251081</v>
+        <v>0.801725108225108</v>
       </c>
       <c r="F573" s="2" t="n">
         <v>1</v>
@@ -17347,7 +17347,7 @@
         </is>
       </c>
       <c r="E583" s="2" t="n">
-        <v>0.5528712233626147</v>
+        <v>0.5528712233626148</v>
       </c>
       <c r="F583" s="2" t="n">
         <v>0</v>
@@ -17434,7 +17434,7 @@
         </is>
       </c>
       <c r="E586" s="2" t="n">
-        <v>0.9333333333333332</v>
+        <v>0.9333333333333335</v>
       </c>
       <c r="F586" s="2" t="n">
         <v>1</v>
@@ -17463,7 +17463,7 @@
         </is>
       </c>
       <c r="E587" s="2" t="n">
-        <v>0.8256363576768099</v>
+        <v>0.8256363576768101</v>
       </c>
       <c r="F587" s="2" t="n">
         <v>0</v>
@@ -17492,7 +17492,7 @@
         </is>
       </c>
       <c r="E588" s="2" t="n">
-        <v>0.39785776520431</v>
+        <v>0.3978577652043099</v>
       </c>
       <c r="F588" s="2" t="n">
         <v>1</v>
@@ -17521,7 +17521,7 @@
         </is>
       </c>
       <c r="E589" s="2" t="n">
-        <v>0.8534189200629879</v>
+        <v>0.8534189200629878</v>
       </c>
       <c r="F589" s="2" t="n">
         <v>1</v>
@@ -17550,7 +17550,7 @@
         </is>
       </c>
       <c r="E590" s="2" t="n">
-        <v>0.8177411490122363</v>
+        <v>0.8177411490122364</v>
       </c>
       <c r="F590" s="2" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
applying matplot.lib to comapre
</commit_message>
<xml_diff>
--- a/final.xlsx
+++ b/final.xlsx
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.7790573593073594</v>
+        <v>0.7790573593073593</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>1</v>
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0.3228667434715821</v>
+        <v>0.3228667434715822</v>
       </c>
       <c r="F17" s="2" t="n">
         <v>1</v>
@@ -2006,7 +2006,7 @@
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>0.5234505175525538</v>
+        <v>0.5234505175525537</v>
       </c>
       <c r="F54" s="2" t="n">
         <v>0</v>
@@ -2586,7 +2586,7 @@
         </is>
       </c>
       <c r="E74" s="2" t="n">
-        <v>0.5965762965105069</v>
+        <v>0.596576296510507</v>
       </c>
       <c r="F74" s="2" t="n">
         <v>0</v>
@@ -2644,7 +2644,7 @@
         </is>
       </c>
       <c r="E76" s="2" t="n">
-        <v>0.6708056247553444</v>
+        <v>0.6708056247553447</v>
       </c>
       <c r="F76" s="2" t="n">
         <v>0</v>
@@ -2760,7 +2760,7 @@
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>0.3934880952380953</v>
+        <v>0.3934880952380952</v>
       </c>
       <c r="F80" s="2" t="n">
         <v>0</v>
@@ -2818,7 +2818,7 @@
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>0.5880358226976868</v>
+        <v>0.5880358226976869</v>
       </c>
       <c r="F82" s="2" t="n">
         <v>0</v>
@@ -3079,7 +3079,7 @@
         </is>
       </c>
       <c r="E91" s="2" t="n">
-        <v>0.8154085497835497</v>
+        <v>0.8154085497835498</v>
       </c>
       <c r="F91" s="2" t="n">
         <v>1</v>
@@ -3862,7 +3862,7 @@
         </is>
       </c>
       <c r="E118" s="2" t="n">
-        <v>0.9705833333333334</v>
+        <v>0.9705833333333335</v>
       </c>
       <c r="F118" s="2" t="n">
         <v>1</v>
@@ -3891,7 +3891,7 @@
         </is>
       </c>
       <c r="E119" s="2" t="n">
-        <v>0.793381953318</v>
+        <v>0.7933819533179998</v>
       </c>
       <c r="F119" s="2" t="n">
         <v>1</v>
@@ -5022,7 +5022,7 @@
         </is>
       </c>
       <c r="E158" s="2" t="n">
-        <v>0.8009922332569391</v>
+        <v>0.8009922332569392</v>
       </c>
       <c r="F158" s="2" t="n">
         <v>0</v>
@@ -5109,7 +5109,7 @@
         </is>
       </c>
       <c r="E161" s="2" t="n">
-        <v>0.784875</v>
+        <v>0.7848749999999999</v>
       </c>
       <c r="F161" s="2" t="n">
         <v>0</v>
@@ -5225,7 +5225,7 @@
         </is>
       </c>
       <c r="E165" s="2" t="n">
-        <v>0.6359596792096791</v>
+        <v>0.6359596792096792</v>
       </c>
       <c r="F165" s="2" t="n">
         <v>1</v>
@@ -5283,7 +5283,7 @@
         </is>
       </c>
       <c r="E167" s="2" t="n">
-        <v>0.09467579365079368</v>
+        <v>0.09467579365079366</v>
       </c>
       <c r="F167" s="2" t="n">
         <v>0</v>
@@ -5631,7 +5631,7 @@
         </is>
       </c>
       <c r="E179" s="2" t="n">
-        <v>0.6844880952380954</v>
+        <v>0.6794880952380954</v>
       </c>
       <c r="F179" s="2" t="n">
         <v>1</v>
@@ -6008,7 +6008,7 @@
         </is>
       </c>
       <c r="E192" s="2" t="n">
-        <v>0.4827796764638869</v>
+        <v>0.482779676463887</v>
       </c>
       <c r="F192" s="2" t="n">
         <v>1</v>
@@ -6124,7 +6124,7 @@
         </is>
       </c>
       <c r="E196" s="2" t="n">
-        <v>0.02558333333333333</v>
+        <v>0.02558333333333334</v>
       </c>
       <c r="F196" s="2" t="n">
         <v>0</v>
@@ -6240,7 +6240,7 @@
         </is>
       </c>
       <c r="E200" s="2" t="n">
-        <v>0.6666135808746061</v>
+        <v>0.666613580874606</v>
       </c>
       <c r="F200" s="2" t="n">
         <v>0</v>
@@ -6675,7 +6675,7 @@
         </is>
       </c>
       <c r="E215" s="2" t="n">
-        <v>0.7010634920634919</v>
+        <v>0.7010634920634921</v>
       </c>
       <c r="F215" s="2" t="n">
         <v>0</v>
@@ -7197,7 +7197,7 @@
         </is>
       </c>
       <c r="E233" s="2" t="n">
-        <v>0.9160651966137885</v>
+        <v>0.9160651966137884</v>
       </c>
       <c r="F233" s="2" t="n">
         <v>1</v>
@@ -7777,7 +7777,7 @@
         </is>
       </c>
       <c r="E253" s="2" t="n">
-        <v>0.2415785533910535</v>
+        <v>0.2415785533910534</v>
       </c>
       <c r="F253" s="2" t="n">
         <v>1</v>
@@ -8618,7 +8618,7 @@
         </is>
       </c>
       <c r="E282" s="2" t="n">
-        <v>0.9439582132748583</v>
+        <v>0.9439582132748585</v>
       </c>
       <c r="F282" s="2" t="n">
         <v>1</v>
@@ -9285,7 +9285,7 @@
         </is>
       </c>
       <c r="E305" s="2" t="n">
-        <v>0.7095952380952382</v>
+        <v>0.7095952380952381</v>
       </c>
       <c r="F305" s="2" t="n">
         <v>1</v>
@@ -9459,7 +9459,7 @@
         </is>
       </c>
       <c r="E311" s="2" t="n">
-        <v>0.07533531746031746</v>
+        <v>0.07533531746031748</v>
       </c>
       <c r="F311" s="2" t="n">
         <v>0</v>
@@ -9865,7 +9865,7 @@
         </is>
       </c>
       <c r="E325" s="2" t="n">
-        <v>0.01165476190476191</v>
+        <v>0.0116547619047619</v>
       </c>
       <c r="F325" s="2" t="n">
         <v>0</v>
@@ -10039,7 +10039,7 @@
         </is>
       </c>
       <c r="E331" s="2" t="n">
-        <v>0.07630357142857144</v>
+        <v>0.07630357142857143</v>
       </c>
       <c r="F331" s="2" t="n">
         <v>0</v>
@@ -10677,7 +10677,7 @@
         </is>
       </c>
       <c r="E353" s="2" t="n">
-        <v>0.8081017666434828</v>
+        <v>0.8081017666434827</v>
       </c>
       <c r="F353" s="2" t="n">
         <v>0</v>
@@ -10793,7 +10793,7 @@
         </is>
       </c>
       <c r="E357" s="2" t="n">
-        <v>0.8958363021387216</v>
+        <v>0.8958363021387215</v>
       </c>
       <c r="F357" s="2" t="n">
         <v>1</v>
@@ -11605,7 +11605,7 @@
         </is>
       </c>
       <c r="E385" s="2" t="n">
-        <v>0.7128478159482416</v>
+        <v>0.7128478159482415</v>
       </c>
       <c r="F385" s="2" t="n">
         <v>0</v>
@@ -12533,7 +12533,7 @@
         </is>
       </c>
       <c r="E417" s="2" t="n">
-        <v>0.7273632668964667</v>
+        <v>0.7273632668964669</v>
       </c>
       <c r="F417" s="2" t="n">
         <v>1</v>
@@ -12794,7 +12794,7 @@
         </is>
       </c>
       <c r="E426" s="2" t="n">
-        <v>0.9555476190476189</v>
+        <v>0.9555476190476191</v>
       </c>
       <c r="F426" s="2" t="n">
         <v>1</v>
@@ -13171,7 +13171,7 @@
         </is>
       </c>
       <c r="E439" s="2" t="n">
-        <v>0.4433062285777805</v>
+        <v>0.4433062285777804</v>
       </c>
       <c r="F439" s="2" t="n">
         <v>0</v>
@@ -13200,7 +13200,7 @@
         </is>
       </c>
       <c r="E440" s="2" t="n">
-        <v>0.903688266952973</v>
+        <v>0.9036882669529729</v>
       </c>
       <c r="F440" s="2" t="n">
         <v>1</v>
@@ -13316,7 +13316,7 @@
         </is>
       </c>
       <c r="E444" s="2" t="n">
-        <v>0.739259388984796</v>
+        <v>0.7392593889847962</v>
       </c>
       <c r="F444" s="2" t="n">
         <v>1</v>
@@ -13374,7 +13374,7 @@
         </is>
       </c>
       <c r="E446" s="2" t="n">
-        <v>0.870545634920635</v>
+        <v>0.8705456349206347</v>
       </c>
       <c r="F446" s="2" t="n">
         <v>1</v>
@@ -13693,7 +13693,7 @@
         </is>
       </c>
       <c r="E457" s="2" t="n">
-        <v>0.5846130952380951</v>
+        <v>0.584613095238095</v>
       </c>
       <c r="F457" s="2" t="n">
         <v>0</v>
@@ -13780,7 +13780,7 @@
         </is>
       </c>
       <c r="E460" s="2" t="n">
-        <v>0.6175337301587301</v>
+        <v>0.6175337301587303</v>
       </c>
       <c r="F460" s="2" t="n">
         <v>0</v>
@@ -14012,7 +14012,7 @@
         </is>
       </c>
       <c r="E468" s="2" t="n">
-        <v>0.9203690476190477</v>
+        <v>0.9203690476190475</v>
       </c>
       <c r="F468" s="2" t="n">
         <v>1</v>
@@ -14041,7 +14041,7 @@
         </is>
       </c>
       <c r="E469" s="2" t="n">
-        <v>0.9838501027246228</v>
+        <v>0.9838501027246227</v>
       </c>
       <c r="F469" s="2" t="n">
         <v>1</v>
@@ -14331,7 +14331,7 @@
         </is>
       </c>
       <c r="E479" s="2" t="n">
-        <v>0.9571834360579561</v>
+        <v>0.9571834360579562</v>
       </c>
       <c r="F479" s="2" t="n">
         <v>1</v>
@@ -14505,7 +14505,7 @@
         </is>
       </c>
       <c r="E485" s="2" t="n">
-        <v>0.7261243525634389</v>
+        <v>0.726124352563439</v>
       </c>
       <c r="F485" s="2" t="n">
         <v>1</v>
@@ -14824,7 +14824,7 @@
         </is>
       </c>
       <c r="E496" s="2" t="n">
-        <v>0.8774583333333333</v>
+        <v>0.8774583333333332</v>
       </c>
       <c r="F496" s="2" t="n">
         <v>1</v>
@@ -14911,7 +14911,7 @@
         </is>
       </c>
       <c r="E499" s="2" t="n">
-        <v>0.8560586923805805</v>
+        <v>0.8560586923805806</v>
       </c>
       <c r="F499" s="2" t="n">
         <v>1</v>
@@ -14940,7 +14940,7 @@
         </is>
       </c>
       <c r="E500" s="2" t="n">
-        <v>0.5786315681444991</v>
+        <v>0.5786315681444992</v>
       </c>
       <c r="F500" s="2" t="n">
         <v>1</v>
@@ -15868,7 +15868,7 @@
         </is>
       </c>
       <c r="E532" s="2" t="n">
-        <v>0.4930892857142859</v>
+        <v>0.4930892857142858</v>
       </c>
       <c r="F532" s="2" t="n">
         <v>0</v>
@@ -16477,7 +16477,7 @@
         </is>
       </c>
       <c r="E553" s="2" t="n">
-        <v>0.7206338074835896</v>
+        <v>0.7206338074835895</v>
       </c>
       <c r="F553" s="2" t="n">
         <v>1</v>
@@ -16651,7 +16651,7 @@
         </is>
       </c>
       <c r="E559" s="2" t="n">
-        <v>0.8435138888888888</v>
+        <v>0.8435138888888889</v>
       </c>
       <c r="F559" s="2" t="n">
         <v>0</v>
@@ -16680,7 +16680,7 @@
         </is>
       </c>
       <c r="E560" s="2" t="n">
-        <v>0.9393333333333331</v>
+        <v>0.9393333333333332</v>
       </c>
       <c r="F560" s="2" t="n">
         <v>1</v>
@@ -16796,7 +16796,7 @@
         </is>
       </c>
       <c r="E564" s="2" t="n">
-        <v>0.5847886527176823</v>
+        <v>0.5847886527176825</v>
       </c>
       <c r="F564" s="2" t="n">
         <v>0</v>
@@ -17231,7 +17231,7 @@
         </is>
       </c>
       <c r="E579" s="2" t="n">
-        <v>0.8401111111111113</v>
+        <v>0.8401111111111114</v>
       </c>
       <c r="F579" s="2" t="n">
         <v>1</v>
@@ -17318,7 +17318,7 @@
         </is>
       </c>
       <c r="E582" s="2" t="n">
-        <v>0.04633333333333333</v>
+        <v>0.04633333333333334</v>
       </c>
       <c r="F582" s="2" t="n">
         <v>0</v>

</xml_diff>